<commit_message>
Database Pekerja: tambah 5 tipe staf (EM, Agronomy Head, Field Supervisor, Warehouse, Water Management Officer) di filter, form & template Excel
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Template-Database-Tenaga-Kerja-HOK.xlsx
+++ b/public/Template-Database-Tenaga-Kerja-HOK.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="231">
   <si>
     <t/>
   </si>
@@ -311,13 +311,28 @@
     <t>FP-B04 · Fingerspot Revo-W</t>
   </si>
   <si>
+    <t>Estate Manager</t>
+  </si>
+  <si>
     <t>Sakit</t>
   </si>
   <si>
     <t>BCA</t>
   </si>
   <si>
+    <t>Agronomy Head</t>
+  </si>
+  <si>
     <t>Tidak hadir</t>
+  </si>
+  <si>
+    <t>Field Supervisor</t>
+  </si>
+  <si>
+    <t>Warehouse Officer</t>
+  </si>
+  <si>
+    <t>Water Management Officer</t>
   </si>
   <si>
     <t>No</t>
@@ -1367,7 +1382,7 @@
   <sheetPr>
     <tabColor rgb="FF9CA3AF"/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="4" width="16" customWidth="1"/>
@@ -1623,18 +1638,20 @@
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="F6" s="7" t="s">
+        <v>98</v>
+      </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
@@ -1646,13 +1663,15 @@
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="F7" s="7" t="s">
+        <v>101</v>
+      </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
@@ -1667,7 +1686,9 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="F8" s="7" t="s">
+        <v>103</v>
+      </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
@@ -1679,6 +1700,48 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1720,52 +1783,52 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>33</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="Q1" s="6" t="s">
         <v>37</v>
@@ -1774,13 +1837,13 @@
         <v>42</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="T1" s="6" t="s">
         <v>38</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="V1" s="6" t="s">
         <v>28</v>
@@ -1791,25 +1854,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>59</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>46</v>
@@ -1827,10 +1890,10 @@
         <v>49</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="O2" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="P2" s="8" t="s">
         <v>52</v>
@@ -1842,16 +1905,16 @@
         <v>58</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="T2" s="8" t="s">
         <v>54</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="V2" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
@@ -1859,25 +1922,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>59</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>46</v>
@@ -1895,10 +1958,10 @@
         <v>49</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="P3" s="8" t="s">
         <v>52</v>
@@ -1910,16 +1973,16 @@
         <v>74</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="T3" s="8" t="s">
         <v>70</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -3509,10 +3572,10 @@
       <formula1>Referensi!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Cek referensi" error="Nilai di luar daftar referensi." sqref="L10:L63">
-      <formula1>Referensi!$F$2:$F$5</formula1>
+      <formula1>Referensi!$F$2:$F$10</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Cek referensi" error="Nilai di luar daftar referensi." sqref="L2:L63">
-      <formula1>Referensi!$F$2:$F$5</formula1>
+      <formula1>Referensi!$F$2:$F$10</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Cek referensi" error="Nilai di luar daftar referensi." sqref="M10:M63">
       <formula1>Referensi!$E$2:$E$5</formula1>
@@ -3575,37 +3638,37 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>44</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>40</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>45</v>
@@ -3622,13 +3685,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>46</v>
@@ -3637,10 +3700,10 @@
         <v>60</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>55</v>
@@ -3658,7 +3721,7 @@
         <v>57</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -3666,13 +3729,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>46</v>
@@ -3681,10 +3744,10 @@
         <v>60</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>71</v>
@@ -3702,7 +3765,7 @@
         <v>73</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -5927,44 +5990,44 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E3" s="7">
         <v>60</v>
@@ -5973,21 +6036,21 @@
         <v>80000</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E4" s="7">
         <v>70</v>
@@ -5996,21 +6059,21 @@
         <v>80000</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E5" s="7">
         <v>80</v>
@@ -6019,21 +6082,21 @@
         <v>80000</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>171</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>166</v>
       </c>
       <c r="E6" s="7">
         <v>120</v>
@@ -6042,21 +6105,21 @@
         <v>80000</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="E7" s="7">
         <v>400</v>
@@ -6065,21 +6128,21 @@
         <v>80000</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E8" s="7">
         <v>150</v>
@@ -6088,21 +6151,21 @@
         <v>90000</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>172</v>
-      </c>
       <c r="D9" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E9" s="7">
         <v>90</v>
@@ -6111,21 +6174,21 @@
         <v>85000</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E10" s="7">
         <v>200</v>
@@ -6134,21 +6197,21 @@
         <v>80000</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E11" s="7">
         <v>120</v>
@@ -6157,21 +6220,21 @@
         <v>95000</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E12" s="7">
         <v>250</v>
@@ -6180,21 +6243,21 @@
         <v>85000</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E13" s="7">
         <v>300</v>
@@ -6203,21 +6266,21 @@
         <v>85000</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E14" s="7">
         <v>180</v>
@@ -6226,21 +6289,21 @@
         <v>90000</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E15" s="7">
         <v>300</v>
@@ -6249,21 +6312,21 @@
         <v>80000</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E16" s="7">
         <v>8</v>
@@ -6272,21 +6335,21 @@
         <v>85000</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="E17" s="7">
         <v>7</v>
@@ -6295,21 +6358,21 @@
         <v>110000</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E18" s="7">
         <v>3</v>
@@ -6318,46 +6381,46 @@
         <v>100000</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>82</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C23" s="12">
         <v>80000</v>
@@ -6369,10 +6432,10 @@
         <v>12000</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>52</v>
@@ -6380,10 +6443,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C24" s="12">
         <v>110000</v>
@@ -6395,10 +6458,10 @@
         <v>16000</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>52</v>
@@ -6406,10 +6469,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C25" s="12">
         <v>75000</v>
@@ -6421,13 +6484,13 @@
         <v>11000</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>